<commit_message>
Added Day 51 (OpenPyXL Library)
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Student Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rahul</t>
+          <t xml:space="preserve">Sai </t>
         </is>
       </c>
       <c r="B3" t="n">

</xml_diff>